<commit_message>
Cap nhat lai cau truc du an
</commit_message>
<xml_diff>
--- a/docs/phân công.xlsx
+++ b/docs/phân công.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="10212" windowHeight="9000"/>
+    <workbookView windowWidth="12431" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,22 +45,23 @@
   </si>
   <si>
     <t>Giai đoạn 9.2: Cài đặt Server cơ bản
-Tạo socket TCP, Bind IP, Port, Listen, Accept client, Mỗi client một thread
+Tạo socket TCP, Bind IP, Port, Listen, Accept client, Mỗi kết nối đến là một thread xử lý riêng biệt.
 Giai đoạn 9.4 – Giao thức (PHÍA SERVER)
-Định dạng thông điệp
-Code hàm: Phân tích yêu cầu, Tạo header file, Tạo thông báo lỗi
+Phân tích DOWNLOAD|filename
+Tạo header FILE|...|SIZE|...
+Tạo thông báo lỗi ERROR|filename|404
 Giai đoạn 9.5 – Download 1 file (SERVER)
-Kiểm tra file tồn tại, Gửi header, Gửi dữ liệu theo buffer, Gửi END_FILE
+Kiểm tra file tồn tại, Gửi header, Gửi dữ liệu theo buffer, File kết thúc bằng filesize
 Giai đoạn 9.6 – Download nhiều file (SERVER)
-Nhận danh sách file, for file in list: gửi lần lượt từng file
+Không cần xử lý danh sách.
+Chỉ cần đảm bảo Accept() liên tục và không bị treo khi có 5-10 kết nối ập vào cùng lúc.
  Giai đoạn 9.7 – Đa luồng phía SERVER
-Mỗi client = 1 thread, Server chính:
-accept → tạo thread → quay lại accept
-Tuyệt đối KHÔNG:
-Mỗi file 1 thread trên cùng socket
+1 Client connection = 1 Thread.
+Luồng chính: while True: accept() -&gt; start_new_thread().Thread tự kết thúc khi client xong việc
 Giai đoạn 9.8 – Xử lý lỗi SERVER
 Client ngắt kết nối giữa chừng, File không tồn tại, 
-Log lỗi, giải phóng thread</t>
+Log lỗi, giải phóng thread. Lỗi từng phần: Nếu File A bị lỗi (404), File B vẫn phải tải bình thường (vì chạy 2 thread khác nhau).
+Timeout: Set timeout cho socket để nếu Server không gửi dữ liệu thì Client tự ngắt thread đó.</t>
   </si>
   <si>
     <t>“Server không treo”
@@ -74,23 +75,20 @@
     <t>Giai đoạn 9.3 – Client cơ bản 
 Tạo socket, Kết nối server, Gửi chuỗi test, Nhận phản hồi
 Giai đoạn 9.4 – Giao thức (PHÍA CLIENT) 
-Tạo request:DOWNLOAD|file1,file2, Gửi đúng format, Nhận &amp; phân tích header
+Client gửi: DOWNLOAD|&lt;tên_file&gt; (Chỉ 1 file mỗi yêu cầu), Gửi đúng format, Nhận &amp; phân tích header
 Giai đoạn 9.5 – Download 1 file (CLIENT)
-Nhận header, Tạo file, Nhận dữ liệu, Ghi file, Nhận END_FILE 
+Nhận header, Gọi receive_file_content(), Ghi file ra disk
 Giai đoạn 9.6 – Download nhiều file (CLIENT)
-Gửi danh sách file, Nhận file tuần tự, Lưu file đúng tên, không ghi đè (đổi tên nếu trùng) 
+Nhận danh sách file từ người dùng (VD: "a.txt, b.pdf").Tách chuỗi thành mảng ['a.txt', 'b.pdf'].Vòng lặp tạo Thread: Với mỗi file trong mảng -&gt;  Khởi tạo 1 Thread mới.Trong mỗi Thread: Tạo socket mới -&gt; Gọi hàm Download 1 file (của Giai đoạn 9.5).
 Giai đoạn 9.7 – Đa luồng phía CLIENT (ĐÚNG BẢN CHẤT)
-👉 Đa luồng ở đây là:
-UI không bị treo
-Hiển thị tiến độ
-Không phải nhiều thread recv socket
-Ví dụ:
-1 thread network
-1 thread UI/progress
+Cơ chế: True Parallelism (Song song thực sự).
+Quy tắc: Mỗi file là một "Worker Thread" riêng biệt.
+Tài nguyên: Mỗi Thread sở hữu 1 Socket riêng (Không dùng chung Socket).
+UI Thread: Một luồng riêng để cập nhật thanh tiến độ tổng hoặc in log ra màn hình mà không bị loạn.
 Giai đoạn 9.8 – Xử lý lỗi CLIENT
 Mất kết nối, File không tồn tại, Thông báo rõ ràng 
 UI đơn giản
-Console hoặc Tkinter, Hiển thị: File đang tải, % tiến độ, Thành công / lỗi</t>
+Console hoặc Tkinter, Hiển thị: File đang tải, % tiến độ, Thành công / lỗi. Test case quan trọng: Nhập 5 file cùng lúc-&gt; Kiểm tra Task Manager xem có đúng là mạng tăng vọt (tải song song) hay không.</t>
   </si>
   <si>
     <t>"UI không treo"
@@ -108,13 +106,19 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -581,142 +585,151 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1251,8 +1264,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="3"/>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="68.8888888888889" customWidth="1"/>
@@ -1273,7 +1286,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="244.8" spans="1:4">
+    <row r="2" ht="331.2" spans="1:4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1283,11 +1296,11 @@
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" ht="302.4" spans="1:4">
+    <row r="3" ht="345.6" spans="1:4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1297,9 +1310,57 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
+    </row>
+    <row r="4" spans="3:3">
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="3:3">
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="3:3">
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="3:3">
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="3:3">
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="3:3">
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" spans="3:3">
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" spans="3:3">
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" spans="3:3">
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" spans="3:3">
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" spans="3:3">
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" spans="3:3">
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" spans="3:3">
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" s="3"/>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>